<commit_message>
Atualiza casos de teste
</commit_message>
<xml_diff>
--- a/docs/casos-de-teste-e2e.xlsx
+++ b/docs/casos-de-teste-e2e.xlsx
@@ -13,17 +13,17 @@
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1776877702" val="982" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1776877702" fixedDigits="0" showNotice="1" showProtection="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1776877702"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1776877702"/>
+      <pm:revision xmlns:pm="smNativeData" day="1776886078" val="982" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1776886078" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1776886078" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1776886078"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="42">
   <si>
     <t>CASO DE TESTE</t>
   </si>
@@ -136,6 +136,65 @@
   <si>
     <t>Emitir alerta:
 "Password é obrigatório"</t>
+  </si>
+  <si>
+    <t>cadastro de usuário com sucesso</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- preencher nome
+- preencher email
+- preencher senha
+- clicar em "Cadastrar"</t>
+  </si>
+  <si>
+    <t>Emitir:
+"Cadastro realizado com sucesso"</t>
+  </si>
+  <si>
+    <t>Cadastro</t>
+  </si>
+  <si>
+    <t>não permite email já registrado</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- preencher nome
+- inserir email já cadastrado
+- preencher senha
+- clicar em "Cadastrar"</t>
+  </si>
+  <si>
+    <t>Emitir alerta:
+"Este email já está sendo usado"</t>
+  </si>
+  <si>
+    <t>exibe erro com nome em branco</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- não preencher nome
+- preencher email
+- preencher senha
+- clicar em "Cadastrar"</t>
+  </si>
+  <si>
+    <t>Emtir alerta:
+"Nome é obrigatório"</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- preencher nome
+- não preencher email 
+- preencher senha
+- clicar em "Cadastrar"</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- preencher nome
+- preencher email 
+- não preencher senha
+- clicar em "Cadastrar"</t>
   </si>
 </sst>
 </file>
@@ -162,7 +221,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776877702" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776886078" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -178,7 +237,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776877702" fgClr="FFFFFF" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1776886078" fgClr="FFFFFF" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -187,7 +246,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -200,7 +259,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -214,7 +273,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -225,7 +284,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -236,7 +295,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -247,7 +317,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -261,18 +331,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -283,29 +342,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -319,7 +356,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -327,19 +364,8 @@
     <fill>
       <patternFill patternType="none"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDEDEDE"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776877702" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="17">
+  <borders count="14">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -355,7 +381,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702"/>
+          <pm:border xmlns:pm="smNativeData" id="1776886078"/>
         </ext>
       </extLst>
     </border>
@@ -374,7 +400,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -398,7 +424,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -422,7 +448,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -445,7 +471,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -468,7 +494,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -486,12 +512,36 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="none">
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -514,7 +564,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -532,74 +582,12 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
+      <bottom style="none">
         <color rgb="FF000000"/>
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -611,10 +599,10 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="thin">
+      <right style="none">
         <color rgb="FF000000"/>
       </right>
-      <top style="none">
+      <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
@@ -622,7 +610,53 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -645,7 +679,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
+          <pm:border xmlns:pm="smNativeData" id="1776886078">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -653,87 +687,13 @@
         </ext>
       </extLst>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776877702"/>
-        </ext>
-      </extLst>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -767,32 +727,38 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,10 +767,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1776877702" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1776886078" count="1">
         <pm:charStyle name="Normal" fontId="0"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1776877702" count="3">
+      <pm:colors xmlns:pm="smNativeData" id="1776886078" count="3">
         <pm:color name="Cor 24" rgb="919191"/>
         <pm:color name="Cor 25" rgb="D9D9D9"/>
         <pm:color name="Cor 26" rgb="DEDEDE"/>
@@ -1084,256 +1050,336 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="29.25" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="67.85" customHeight="1">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="63.70" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="63.45" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9"/>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
+      <c r="A9" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10"/>
-      <c r="B10"/>
-      <c r="C10"/>
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
+      <c r="A10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11"/>
-      <c r="B11"/>
-      <c r="C11"/>
-      <c r="D11"/>
-      <c r="E11"/>
-      <c r="F11"/>
-      <c r="G11"/>
-      <c r="H11"/>
+      <c r="A11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12"/>
-      <c r="B12"/>
-      <c r="C12"/>
-      <c r="D12"/>
-      <c r="E12"/>
-      <c r="F12"/>
-      <c r="G12"/>
-      <c r="H12"/>
+      <c r="A12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13"/>
-      <c r="B13"/>
-      <c r="C13"/>
-      <c r="D13"/>
-      <c r="E13"/>
-      <c r="F13"/>
-      <c r="G13"/>
-      <c r="H13"/>
+      <c r="A13" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14"/>
-      <c r="B14"/>
-      <c r="C14"/>
-      <c r="D14"/>
-      <c r="E14"/>
-      <c r="F14"/>
-      <c r="G14"/>
-      <c r="H14"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" ht="74.75" customHeight="1">
       <c r="A15"/>
@@ -1396,514 +1442,540 @@
       <c r="H20"/>
     </row>
     <row r="21" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A21" s="18"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
+      <c r="A21"/>
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
+      <c r="F21"/>
+      <c r="G21"/>
+      <c r="H21"/>
     </row>
     <row r="22" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A22" s="18"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
+      <c r="A22"/>
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22"/>
+      <c r="H22"/>
     </row>
     <row r="23" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A23" s="18"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
+      <c r="A23"/>
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23"/>
     </row>
     <row r="24" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A24" s="18"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
+      <c r="A24"/>
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+      <c r="E24"/>
+      <c r="F24"/>
+      <c r="G24"/>
+      <c r="H24"/>
     </row>
     <row r="25" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A25" s="22"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
+      <c r="A25"/>
+      <c r="B25"/>
+      <c r="C25"/>
+      <c r="D25"/>
+      <c r="E25"/>
+      <c r="F25"/>
+      <c r="G25"/>
+      <c r="H25"/>
     </row>
     <row r="26" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A26" s="22"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
+      <c r="A26"/>
+      <c r="B26"/>
+      <c r="C26"/>
+      <c r="D26"/>
+      <c r="E26"/>
+      <c r="F26"/>
+      <c r="G26"/>
+      <c r="H26"/>
     </row>
     <row r="27" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A27" s="22"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
+      <c r="A27"/>
+      <c r="B27"/>
+      <c r="C27"/>
+      <c r="D27"/>
+      <c r="E27"/>
+      <c r="F27"/>
+      <c r="G27"/>
+      <c r="H27"/>
     </row>
     <row r="28" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A28" s="22"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
+      <c r="A28"/>
+      <c r="B28"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
     </row>
     <row r="29" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A29" s="22"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
+      <c r="A29"/>
+      <c r="B29"/>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29"/>
+      <c r="F29"/>
+      <c r="G29"/>
+      <c r="H29"/>
     </row>
     <row r="30" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A30" s="22"/>
-      <c r="B30" s="23"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
+      <c r="A30"/>
+      <c r="B30"/>
+      <c r="C30"/>
+      <c r="D30"/>
+      <c r="E30"/>
+      <c r="F30"/>
+      <c r="G30"/>
+      <c r="H30"/>
     </row>
     <row r="31" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A31" s="22"/>
-      <c r="B31" s="23"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
+      <c r="A31"/>
+      <c r="B31"/>
+      <c r="C31"/>
+      <c r="D31"/>
+      <c r="E31"/>
+      <c r="F31"/>
+      <c r="G31"/>
+      <c r="H31"/>
     </row>
     <row r="32" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A32" s="22"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
+      <c r="A32"/>
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="E32"/>
+      <c r="F32"/>
+      <c r="G32"/>
+      <c r="H32"/>
     </row>
     <row r="33" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A33" s="22"/>
-      <c r="B33" s="23"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
+      <c r="A33"/>
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="H33"/>
     </row>
     <row r="34" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A34" s="22"/>
-      <c r="B34" s="23"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
+      <c r="A34"/>
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="E34"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="H34"/>
     </row>
     <row r="35" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A35" s="1"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
+      <c r="A35"/>
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="E35"/>
+      <c r="F35"/>
+      <c r="G35"/>
+      <c r="H35"/>
     </row>
     <row r="36" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A36" s="1"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
+      <c r="A36"/>
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="E36"/>
+      <c r="F36"/>
+      <c r="G36"/>
+      <c r="H36"/>
     </row>
     <row r="37" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A37" s="1"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
+      <c r="A37"/>
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37"/>
+      <c r="F37"/>
+      <c r="G37"/>
+      <c r="H37"/>
     </row>
     <row r="38" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A38" s="3"/>
-      <c r="C38" s="17"/>
+      <c r="A38"/>
+      <c r="B38"/>
+      <c r="C38"/>
     </row>
     <row r="39" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A39" s="3"/>
-      <c r="C39" s="17"/>
+      <c r="A39"/>
+      <c r="B39"/>
+      <c r="C39"/>
     </row>
     <row r="40" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A40" s="3"/>
-      <c r="C40" s="17"/>
+      <c r="A40"/>
+      <c r="B40"/>
+      <c r="C40"/>
     </row>
     <row r="41" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A41" s="3"/>
-      <c r="C41" s="17"/>
+      <c r="A41"/>
+      <c r="B41"/>
+      <c r="C41"/>
     </row>
     <row r="42" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A42" s="3"/>
-      <c r="C42" s="17"/>
+      <c r="A42"/>
+      <c r="B42"/>
+      <c r="C42"/>
     </row>
     <row r="43" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A43" s="3"/>
-      <c r="C43" s="17"/>
+      <c r="A43"/>
+      <c r="B43"/>
+      <c r="C43"/>
     </row>
     <row r="44" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A44" s="3"/>
-      <c r="C44" s="17"/>
+      <c r="A44"/>
+      <c r="B44"/>
+      <c r="C44"/>
     </row>
     <row r="45" spans="1:3">
-      <c r="A45" s="3"/>
-      <c r="C45" s="4"/>
+      <c r="A45"/>
+      <c r="B45"/>
+      <c r="C45"/>
     </row>
     <row r="46" spans="1:3">
-      <c r="A46" s="3"/>
-      <c r="C46" s="4"/>
+      <c r="A46"/>
+      <c r="B46"/>
+      <c r="C46"/>
     </row>
     <row r="47" spans="1:3">
-      <c r="A47" s="3"/>
-      <c r="C47" s="4"/>
+      <c r="A47"/>
+      <c r="B47"/>
+      <c r="C47"/>
     </row>
     <row r="48" spans="1:3">
-      <c r="A48" s="3"/>
-      <c r="C48" s="4"/>
+      <c r="A48"/>
+      <c r="B48"/>
+      <c r="C48"/>
     </row>
     <row r="49" spans="1:3">
-      <c r="A49" s="3"/>
-      <c r="C49" s="4"/>
+      <c r="A49"/>
+      <c r="B49"/>
+      <c r="C49"/>
     </row>
     <row r="50" spans="1:3">
-      <c r="A50" s="3"/>
-      <c r="C50" s="4"/>
+      <c r="A50"/>
+      <c r="B50"/>
+      <c r="C50"/>
     </row>
     <row r="51" spans="1:3">
-      <c r="A51" s="3"/>
-      <c r="C51" s="4"/>
+      <c r="A51"/>
+      <c r="B51"/>
+      <c r="C51"/>
     </row>
     <row r="52" spans="1:3">
-      <c r="A52" s="3"/>
-      <c r="C52" s="4"/>
+      <c r="A52"/>
+      <c r="B52"/>
+      <c r="C52"/>
     </row>
     <row r="53" spans="1:3">
-      <c r="A53" s="3"/>
-      <c r="C53" s="4"/>
+      <c r="A53"/>
+      <c r="B53"/>
+      <c r="C53"/>
     </row>
     <row r="54" spans="1:3">
-      <c r="A54" s="3"/>
-      <c r="C54" s="4"/>
+      <c r="A54"/>
+      <c r="B54"/>
+      <c r="C54"/>
     </row>
     <row r="55" spans="1:3">
-      <c r="A55" s="3"/>
-      <c r="C55" s="4"/>
+      <c r="A55"/>
+      <c r="B55"/>
+      <c r="C55"/>
     </row>
     <row r="56" spans="1:3">
-      <c r="A56" s="3"/>
-      <c r="C56" s="4"/>
+      <c r="A56"/>
+      <c r="B56"/>
+      <c r="C56"/>
     </row>
     <row r="57" spans="1:3">
-      <c r="A57" s="3"/>
-      <c r="C57" s="4"/>
+      <c r="A57"/>
+      <c r="B57"/>
+      <c r="C57"/>
     </row>
     <row r="58" spans="1:3">
-      <c r="A58" s="3"/>
-      <c r="C58" s="4"/>
+      <c r="A58"/>
+      <c r="B58"/>
+      <c r="C58"/>
     </row>
     <row r="59" spans="1:3">
-      <c r="A59" s="3"/>
-      <c r="C59" s="4"/>
+      <c r="A59"/>
+      <c r="B59"/>
+      <c r="C59"/>
     </row>
     <row r="60" spans="1:3">
-      <c r="A60" s="3"/>
-      <c r="C60" s="4"/>
+      <c r="A60"/>
+      <c r="B60"/>
+      <c r="C60"/>
     </row>
     <row r="61" spans="1:3">
-      <c r="A61" s="3"/>
-      <c r="C61" s="4"/>
+      <c r="A61"/>
+      <c r="B61"/>
+      <c r="C61"/>
     </row>
     <row r="62" spans="1:3">
-      <c r="A62" s="3"/>
-      <c r="C62" s="4"/>
+      <c r="A62"/>
+      <c r="B62"/>
+      <c r="C62"/>
     </row>
     <row r="63" spans="1:1">
-      <c r="A63" s="3"/>
+      <c r="A63"/>
     </row>
     <row r="64" spans="1:1">
-      <c r="A64" s="3"/>
+      <c r="A64"/>
     </row>
     <row r="65" spans="1:1">
-      <c r="A65" s="3"/>
+      <c r="A65"/>
     </row>
     <row r="66" spans="1:1">
-      <c r="A66" s="3"/>
+      <c r="A66"/>
     </row>
     <row r="67" spans="1:1">
-      <c r="A67" s="3"/>
+      <c r="A67"/>
     </row>
     <row r="68" spans="1:1">
-      <c r="A68" s="3"/>
+      <c r="A68"/>
     </row>
     <row r="69" spans="1:1">
-      <c r="A69" s="3"/>
+      <c r="A69"/>
     </row>
     <row r="70" spans="1:1">
-      <c r="A70" s="3"/>
+      <c r="A70"/>
     </row>
     <row r="71" spans="1:1">
-      <c r="A71" s="3"/>
+      <c r="A71"/>
     </row>
     <row r="72" spans="1:1">
-      <c r="A72" s="3"/>
+      <c r="A72" s="1"/>
     </row>
     <row r="73" spans="1:1">
-      <c r="A73" s="3"/>
+      <c r="A73" s="1"/>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="3"/>
+      <c r="A74" s="1"/>
     </row>
     <row r="75" spans="1:1">
-      <c r="A75" s="3"/>
+      <c r="A75" s="1"/>
     </row>
     <row r="76" spans="1:1">
-      <c r="A76" s="3"/>
+      <c r="A76" s="1"/>
     </row>
     <row r="77" spans="1:1">
-      <c r="A77" s="3"/>
+      <c r="A77" s="1"/>
     </row>
     <row r="78" spans="1:1">
-      <c r="A78" s="3"/>
+      <c r="A78" s="1"/>
     </row>
     <row r="79" spans="1:1">
-      <c r="A79" s="3"/>
+      <c r="A79" s="1"/>
     </row>
     <row r="80" spans="1:1">
-      <c r="A80" s="3"/>
+      <c r="A80" s="1"/>
     </row>
     <row r="81" spans="1:1">
-      <c r="A81" s="3"/>
+      <c r="A81" s="1"/>
     </row>
     <row r="82" spans="1:1">
-      <c r="A82" s="3"/>
+      <c r="A82" s="1"/>
     </row>
     <row r="83" spans="1:1">
-      <c r="A83" s="3"/>
+      <c r="A83" s="1"/>
     </row>
     <row r="84" spans="1:1">
-      <c r="A84" s="3"/>
+      <c r="A84" s="1"/>
     </row>
     <row r="85" spans="1:1">
-      <c r="A85" s="3"/>
+      <c r="A85" s="1"/>
     </row>
     <row r="86" spans="1:1">
-      <c r="A86" s="3"/>
+      <c r="A86" s="1"/>
     </row>
     <row r="87" spans="1:1">
-      <c r="A87" s="3"/>
+      <c r="A87" s="1"/>
     </row>
     <row r="88" spans="1:1">
-      <c r="A88" s="3"/>
+      <c r="A88" s="1"/>
     </row>
     <row r="89" spans="1:1">
-      <c r="A89" s="3"/>
+      <c r="A89" s="1"/>
     </row>
     <row r="90" spans="1:1">
-      <c r="A90" s="3"/>
+      <c r="A90" s="1"/>
     </row>
     <row r="91" spans="1:1">
-      <c r="A91" s="3"/>
+      <c r="A91" s="1"/>
     </row>
     <row r="92" spans="1:1">
-      <c r="A92" s="3"/>
+      <c r="A92" s="1"/>
     </row>
     <row r="93" spans="1:1">
-      <c r="A93" s="3"/>
+      <c r="A93" s="1"/>
     </row>
     <row r="94" spans="1:1">
-      <c r="A94" s="3"/>
+      <c r="A94" s="1"/>
     </row>
     <row r="95" spans="1:1">
-      <c r="A95" s="3"/>
+      <c r="A95" s="1"/>
     </row>
     <row r="96" spans="1:1">
-      <c r="A96" s="3"/>
+      <c r="A96" s="1"/>
     </row>
     <row r="97" spans="1:1">
-      <c r="A97" s="3"/>
+      <c r="A97" s="1"/>
     </row>
     <row r="98" spans="1:1">
-      <c r="A98" s="3"/>
+      <c r="A98" s="1"/>
     </row>
     <row r="99" spans="1:1">
-      <c r="A99" s="3"/>
+      <c r="A99" s="1"/>
     </row>
     <row r="100" spans="1:1">
-      <c r="A100" s="3"/>
+      <c r="A100" s="1"/>
     </row>
     <row r="101" spans="1:1">
-      <c r="A101" s="3"/>
+      <c r="A101" s="1"/>
     </row>
     <row r="102" spans="1:1">
-      <c r="A102" s="3"/>
+      <c r="A102" s="1"/>
     </row>
     <row r="103" spans="1:1">
-      <c r="A103" s="3"/>
+      <c r="A103" s="1"/>
     </row>
     <row r="104" spans="1:1">
-      <c r="A104" s="3"/>
+      <c r="A104" s="1"/>
     </row>
     <row r="105" spans="1:1">
-      <c r="A105" s="3"/>
+      <c r="A105" s="1"/>
     </row>
     <row r="106" spans="1:1">
-      <c r="A106" s="3"/>
+      <c r="A106" s="1"/>
     </row>
     <row r="107" spans="1:1">
-      <c r="A107" s="3"/>
+      <c r="A107" s="1"/>
     </row>
     <row r="108" spans="1:1">
-      <c r="A108" s="3"/>
+      <c r="A108" s="1"/>
     </row>
     <row r="109" spans="1:1">
-      <c r="A109" s="3"/>
+      <c r="A109" s="1"/>
     </row>
     <row r="110" spans="1:1">
-      <c r="A110" s="3"/>
+      <c r="A110" s="1"/>
     </row>
     <row r="111" spans="1:1">
-      <c r="A111" s="3"/>
+      <c r="A111" s="1"/>
     </row>
     <row r="112" spans="1:1">
-      <c r="A112" s="3"/>
+      <c r="A112" s="1"/>
     </row>
     <row r="113" spans="1:1">
-      <c r="A113" s="3"/>
+      <c r="A113" s="1"/>
     </row>
     <row r="114" spans="1:1">
-      <c r="A114" s="3"/>
+      <c r="A114" s="1"/>
     </row>
     <row r="115" spans="1:1">
-      <c r="A115" s="3"/>
+      <c r="A115" s="1"/>
     </row>
     <row r="116" spans="1:1">
-      <c r="A116" s="3"/>
+      <c r="A116" s="1"/>
     </row>
     <row r="117" spans="1:1">
-      <c r="A117" s="3"/>
+      <c r="A117" s="1"/>
     </row>
     <row r="118" spans="1:1">
-      <c r="A118" s="3"/>
+      <c r="A118" s="1"/>
     </row>
     <row r="119" spans="1:1">
-      <c r="A119" s="3"/>
+      <c r="A119" s="1"/>
     </row>
     <row r="120" spans="1:1">
-      <c r="A120" s="3"/>
+      <c r="A120" s="1"/>
     </row>
     <row r="121" spans="1:1">
-      <c r="A121" s="3"/>
+      <c r="A121" s="1"/>
     </row>
     <row r="122" spans="1:1">
-      <c r="A122" s="3"/>
+      <c r="A122" s="1"/>
     </row>
     <row r="123" spans="1:1">
-      <c r="A123" s="3"/>
+      <c r="A123" s="1"/>
     </row>
     <row r="124" spans="1:1">
-      <c r="A124" s="3"/>
+      <c r="A124" s="1"/>
     </row>
     <row r="125" spans="1:1">
-      <c r="A125" s="3"/>
+      <c r="A125" s="1"/>
     </row>
     <row r="126" spans="1:1">
-      <c r="A126" s="3"/>
+      <c r="A126" s="1"/>
     </row>
     <row r="127" spans="1:1">
-      <c r="A127" s="3"/>
+      <c r="A127" s="1"/>
     </row>
     <row r="128" spans="1:1">
-      <c r="A128" s="3"/>
+      <c r="A128" s="1"/>
     </row>
     <row r="129" spans="1:1">
-      <c r="A129" s="3"/>
+      <c r="A129" s="1"/>
     </row>
     <row r="130" spans="1:1">
-      <c r="A130" s="3"/>
+      <c r="A130" s="1"/>
     </row>
     <row r="131" spans="1:1">
-      <c r="A131" s="3"/>
+      <c r="A131" s="1"/>
     </row>
     <row r="132" spans="1:1">
-      <c r="A132" s="3"/>
+      <c r="A132" s="1"/>
     </row>
     <row r="133" spans="1:1">
-      <c r="A133" s="3"/>
+      <c r="A133" s="1"/>
     </row>
     <row r="134" spans="1:1">
-      <c r="A134" s="3"/>
+      <c r="A134" s="1"/>
     </row>
     <row r="135" spans="1:1">
-      <c r="A135" s="3"/>
+      <c r="A135" s="1"/>
     </row>
     <row r="136" spans="1:1">
-      <c r="A136" s="3"/>
+      <c r="A136" s="1"/>
     </row>
     <row r="137" spans="1:1">
-      <c r="A137" s="3"/>
+      <c r="A137" s="1"/>
     </row>
     <row r="138" spans="1:1">
-      <c r="A138" s="3"/>
+      <c r="A138" s="1"/>
     </row>
     <row r="139" spans="1:1">
-      <c r="A139" s="3"/>
+      <c r="A139" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A14:H14"/>
   </mergeCells>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776877702" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1776886078" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1912,16 +1984,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776877702" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776877702" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1776877702" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1776877702" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1776886078" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1776886078" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1776886078" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1776886078" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776877702" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776886078" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Adiciona fluxo de compras e atualiza README
</commit_message>
<xml_diff>
--- a/docs/casos-de-teste-e2e.xlsx
+++ b/docs/casos-de-teste-e2e.xlsx
@@ -13,17 +13,17 @@
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1776886078" val="982" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1776886078" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1776886078" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1776886078"/>
+      <pm:revision xmlns:pm="smNativeData" day="1777497327" val="982" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1777497327" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1777497327" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1777497327"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="64">
   <si>
     <t>CASO DE TESTE</t>
   </si>
@@ -195,6 +195,92 @@
 - preencher email 
 - não preencher senha
 - clicar em "Cadastrar"</t>
+  </si>
+  <si>
+    <t>adiciona produto na lista pela página inicial</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- logar conta
+- selecionar produto
+- clicar em "Adicionar a lista"</t>
+  </si>
+  <si>
+    <t>produto é adicionado e usuário é direcionado à pagina "lista de compras"</t>
+  </si>
+  <si>
+    <t>Fluxo de Compras</t>
+  </si>
+  <si>
+    <t>acessa lista de compras</t>
+  </si>
+  <si>
+    <t>-acessar o site
+-logar conta
+-clicar em "Lista de Compras"</t>
+  </si>
+  <si>
+    <t>usuario é direcionado à lista de compras</t>
+  </si>
+  <si>
+    <t>limpa a lista</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- logar conta
+- acessar lista de compras
+- clicar "Limpar lista"</t>
+  </si>
+  <si>
+    <t>exclui os produtos e mostra a mensagem:
+"Seu carrinho está vazio"</t>
+  </si>
+  <si>
+    <t>da lista de compras retorna à pagina inicial</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- logar conta
+- acessar lista de compras
+- clicar "Página Inicial"</t>
+  </si>
+  <si>
+    <t>usuario é direcionado à página inicial</t>
+  </si>
+  <si>
+    <t>exibe detalhes do produto selecionado</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- logar conta
+- clicar em "Detalhes" no produto escolhido</t>
+  </si>
+  <si>
+    <t>usuario é direcionado à pagina de detalhes do produto escolhido</t>
+  </si>
+  <si>
+    <t>adiciona produto na lista pela página de detalhes</t>
+  </si>
+  <si>
+    <t>- acessar site
+- logar conta
+- ver detalhes do produto
+- clicar em "Adicionar a lista"</t>
+  </si>
+  <si>
+    <t>produto é adicionado e usuário é direcionado a pagina "lista de compras"</t>
+  </si>
+  <si>
+    <t>da pagina de detalhes retorna à pagina inicial</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- logar conta
+- ver detalhes do produto
+- clicar em "Voltar"</t>
+  </si>
+  <si>
+    <t>retorna à pagina inicial</t>
   </si>
 </sst>
 </file>
@@ -213,7 +299,7 @@
     <numFmt numFmtId="164" formatCode="000"/>
     <numFmt numFmtId="49" formatCode="@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -221,7 +307,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776886078" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777497327" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -237,7 +323,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1776886078" fgClr="FFFFFF" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777497327" fgClr="FFFFFF" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -245,8 +331,23 @@
         </ext>
       </extLst>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:charSpec xmlns:pm="smNativeData" id="1777497327" ulstyle="none" kern="1">
+            <pm:latin face="Arial" sz="220" lang="default"/>
+            <pm:cs face="Times New Roman" sz="220" lang="default"/>
+            <pm:ea face="SimSun" sz="220" lang="default"/>
+          </pm:charSpec>
+        </ext>
+      </extLst>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -259,7 +360,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -273,7 +374,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -284,7 +385,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -295,7 +396,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -306,7 +407,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -317,7 +418,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -331,7 +432,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -342,7 +443,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -356,7 +457,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1776886078" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -364,8 +465,66 @@
     <fill>
       <patternFill patternType="none"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEDEDE"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEDEDE"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="20">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -381,7 +540,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078"/>
+          <pm:border xmlns:pm="smNativeData" id="1777497327"/>
         </ext>
       </extLst>
     </border>
@@ -400,7 +559,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -424,7 +583,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -448,7 +607,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -471,7 +630,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -494,7 +653,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -517,7 +676,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -541,7 +700,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -564,7 +723,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -587,7 +746,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -610,7 +769,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -633,7 +792,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -656,7 +815,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -679,9 +838,138 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1776886078">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777497327"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777497327"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1777497327">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -691,14 +979,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -721,32 +1012,26 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -754,10 +1039,49 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="20" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -767,10 +1091,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1776886078" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1777497327" count="1">
         <pm:charStyle name="Normal" fontId="0"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1776886078" count="3">
+      <pm:colors xmlns:pm="smNativeData" id="1777497327" count="3">
         <pm:color name="Cor 24" rgb="919191"/>
         <pm:color name="Cor 25" rgb="D9D9D9"/>
         <pm:color name="Cor 26" rgb="DEDEDE"/>
@@ -1036,936 +1360,982 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H139"/>
+  <dimension ref="A1:XFD139"/>
   <sheetFormatPr baseColWidth="9" defaultColWidth="10.000000" defaultRowHeight="13.45"/>
   <cols>
-    <col min="1" max="1" width="15.207207" customWidth="1"/>
-    <col min="2" max="2" width="25.963964" customWidth="1"/>
-    <col min="3" max="3" width="31.873874" customWidth="1"/>
-    <col min="4" max="4" width="23.225225" customWidth="1"/>
-    <col min="5" max="5" width="26.333333" customWidth="1"/>
-    <col min="6" max="6" width="17.702703" customWidth="1"/>
-    <col min="7" max="7" width="19.306306" customWidth="1"/>
-    <col min="8" max="8" width="15.378378" customWidth="1"/>
+    <col min="1" max="1" width="16.945946" customWidth="1" style="0"/>
+    <col min="2" max="2" width="25.963964" customWidth="1" style="0"/>
+    <col min="3" max="3" width="31.873874" customWidth="1" style="0"/>
+    <col min="4" max="4" width="23.225225" customWidth="1" style="0"/>
+    <col min="5" max="5" width="26.333333" customWidth="1" style="0"/>
+    <col min="6" max="6" width="17.702703" customWidth="1" style="0"/>
+    <col min="7" max="7" width="20.846847" customWidth="1" style="0"/>
+    <col min="8" max="8" width="15.378378" customWidth="1" style="0"/>
+    <col min="9" max="16384" width="10.000000" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29.25" customHeight="1">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:16384" ht="29.25" customHeight="1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="67.85" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="63.70" customHeight="1">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="32" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="63.45" customHeight="1">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="A8" s="33"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="32" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="34" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="32" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="H13" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="2"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
     </row>
     <row r="15" spans="1:8" ht="74.75" customHeight="1">
-      <c r="A15"/>
-      <c r="B15"/>
-      <c r="C15"/>
-      <c r="D15"/>
-      <c r="E15"/>
-      <c r="F15"/>
-      <c r="G15"/>
-      <c r="H15"/>
+      <c r="A15" s="29" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="59.60" customHeight="1">
-      <c r="A16"/>
-      <c r="B16"/>
-      <c r="C16"/>
-      <c r="D16"/>
-      <c r="E16"/>
-      <c r="F16"/>
-      <c r="G16"/>
-      <c r="H16"/>
+      <c r="A16" s="30" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17"/>
-      <c r="B17"/>
-      <c r="C17"/>
-      <c r="D17"/>
-      <c r="E17"/>
-      <c r="F17"/>
-      <c r="G17"/>
-      <c r="H17"/>
+      <c r="A17" s="30" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="55.40" customHeight="1">
-      <c r="A18"/>
-      <c r="B18"/>
-      <c r="C18"/>
-      <c r="D18"/>
-      <c r="E18"/>
-      <c r="F18"/>
-      <c r="G18"/>
-      <c r="H18"/>
+      <c r="A18" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A19"/>
-      <c r="B19"/>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-      <c r="G19"/>
-      <c r="H19"/>
+      <c r="A19" s="30" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20"/>
-      <c r="B20"/>
-      <c r="C20"/>
-      <c r="D20"/>
-      <c r="E20"/>
-      <c r="F20"/>
-      <c r="G20"/>
-      <c r="H20"/>
+      <c r="A20" s="30" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
+      <c r="A21" s="30" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
+      <c r="A22" s="21"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
     </row>
     <row r="23" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A23"/>
-      <c r="B23"/>
-      <c r="C23"/>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23"/>
+      <c r="A23" s="21"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
     </row>
     <row r="24" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A24"/>
-      <c r="B24"/>
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-      <c r="H24"/>
+      <c r="A24" s="25"/>
     </row>
     <row r="25" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25"/>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25"/>
-      <c r="H25"/>
+      <c r="A25" s="25"/>
     </row>
     <row r="26" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
+      <c r="A26" s="25"/>
     </row>
     <row r="27" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A27"/>
-      <c r="B27"/>
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27"/>
-      <c r="H27"/>
+      <c r="A27" s="21"/>
     </row>
     <row r="28" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A28"/>
-      <c r="B28"/>
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28"/>
-      <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
+      <c r="A28" s="21"/>
     </row>
     <row r="29" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
+      <c r="A29" s="21"/>
     </row>
     <row r="30" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30"/>
-      <c r="G30"/>
-      <c r="H30"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31"/>
-      <c r="G31"/>
-      <c r="H31"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-      <c r="G32"/>
-      <c r="H32"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
     </row>
     <row r="33" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-      <c r="G33"/>
-      <c r="H33"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
     </row>
     <row r="34" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-      <c r="F34"/>
-      <c r="G34"/>
-      <c r="H34"/>
+      <c r="A34" s="14"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
     </row>
     <row r="35" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-      <c r="F35"/>
-      <c r="G35"/>
-      <c r="H35"/>
+      <c r="A35" s="1"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
     </row>
     <row r="36" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
-      <c r="G36"/>
-      <c r="H36"/>
+      <c r="A36" s="1"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
     </row>
     <row r="37" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
+      <c r="A37" s="1"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
     </row>
     <row r="38" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38"/>
+      <c r="A38" s="3"/>
+      <c r="C38" s="13"/>
     </row>
     <row r="39" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A39"/>
-      <c r="B39"/>
-      <c r="C39"/>
+      <c r="A39" s="3"/>
+      <c r="C39" s="13"/>
     </row>
     <row r="40" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A40"/>
-      <c r="B40"/>
-      <c r="C40"/>
+      <c r="A40" s="3"/>
+      <c r="C40" s="13"/>
     </row>
     <row r="41" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A41"/>
-      <c r="B41"/>
-      <c r="C41"/>
+      <c r="A41" s="3"/>
+      <c r="C41" s="13"/>
     </row>
     <row r="42" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A42"/>
-      <c r="B42"/>
-      <c r="C42"/>
+      <c r="A42" s="3"/>
+      <c r="C42" s="13"/>
     </row>
     <row r="43" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A43"/>
-      <c r="B43"/>
-      <c r="C43"/>
+      <c r="A43" s="3"/>
+      <c r="C43" s="13"/>
     </row>
     <row r="44" spans="1:3" ht="53.90" customHeight="1">
-      <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
+      <c r="A44" s="3"/>
+      <c r="C44" s="13"/>
     </row>
     <row r="45" spans="1:3">
-      <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
+      <c r="A45" s="3"/>
+      <c r="C45" s="4"/>
     </row>
     <row r="46" spans="1:3">
-      <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
+      <c r="A46" s="3"/>
+      <c r="C46" s="4"/>
     </row>
     <row r="47" spans="1:3">
-      <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
+      <c r="A47" s="3"/>
+      <c r="C47" s="4"/>
     </row>
     <row r="48" spans="1:3">
-      <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
+      <c r="A48" s="3"/>
+      <c r="C48" s="4"/>
     </row>
     <row r="49" spans="1:3">
-      <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
+      <c r="A49" s="3"/>
+      <c r="C49" s="4"/>
     </row>
     <row r="50" spans="1:3">
-      <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
+      <c r="A50" s="3"/>
+      <c r="C50" s="4"/>
     </row>
     <row r="51" spans="1:3">
-      <c r="A51"/>
-      <c r="B51"/>
-      <c r="C51"/>
+      <c r="A51" s="3"/>
+      <c r="C51" s="4"/>
     </row>
     <row r="52" spans="1:3">
-      <c r="A52"/>
-      <c r="B52"/>
-      <c r="C52"/>
+      <c r="A52" s="3"/>
+      <c r="C52" s="4"/>
     </row>
     <row r="53" spans="1:3">
-      <c r="A53"/>
-      <c r="B53"/>
-      <c r="C53"/>
+      <c r="A53" s="3"/>
+      <c r="C53" s="4"/>
     </row>
     <row r="54" spans="1:3">
-      <c r="A54"/>
-      <c r="B54"/>
-      <c r="C54"/>
+      <c r="A54" s="3"/>
+      <c r="C54" s="4"/>
     </row>
     <row r="55" spans="1:3">
-      <c r="A55"/>
-      <c r="B55"/>
-      <c r="C55"/>
+      <c r="A55" s="3"/>
+      <c r="C55" s="4"/>
     </row>
     <row r="56" spans="1:3">
-      <c r="A56"/>
-      <c r="B56"/>
-      <c r="C56"/>
+      <c r="A56" s="3"/>
+      <c r="C56" s="4"/>
     </row>
     <row r="57" spans="1:3">
-      <c r="A57"/>
-      <c r="B57"/>
-      <c r="C57"/>
+      <c r="A57" s="3"/>
+      <c r="C57" s="4"/>
     </row>
     <row r="58" spans="1:3">
-      <c r="A58"/>
-      <c r="B58"/>
-      <c r="C58"/>
+      <c r="A58" s="3"/>
+      <c r="C58" s="4"/>
     </row>
     <row r="59" spans="1:3">
-      <c r="A59"/>
-      <c r="B59"/>
-      <c r="C59"/>
+      <c r="A59" s="3"/>
+      <c r="C59" s="4"/>
     </row>
     <row r="60" spans="1:3">
-      <c r="A60"/>
-      <c r="B60"/>
-      <c r="C60"/>
+      <c r="A60" s="3"/>
+      <c r="C60" s="4"/>
     </row>
     <row r="61" spans="1:3">
-      <c r="A61"/>
-      <c r="B61"/>
-      <c r="C61"/>
+      <c r="A61" s="3"/>
+      <c r="C61" s="4"/>
     </row>
     <row r="62" spans="1:3">
-      <c r="A62"/>
-      <c r="B62"/>
-      <c r="C62"/>
+      <c r="A62" s="3"/>
+      <c r="C62" s="4"/>
     </row>
     <row r="63" spans="1:1">
-      <c r="A63"/>
+      <c r="A63" s="3"/>
     </row>
     <row r="64" spans="1:1">
-      <c r="A64"/>
+      <c r="A64" s="3"/>
     </row>
     <row r="65" spans="1:1">
-      <c r="A65"/>
+      <c r="A65" s="3"/>
     </row>
     <row r="66" spans="1:1">
-      <c r="A66"/>
+      <c r="A66" s="3"/>
     </row>
     <row r="67" spans="1:1">
-      <c r="A67"/>
+      <c r="A67" s="3"/>
     </row>
     <row r="68" spans="1:1">
-      <c r="A68"/>
+      <c r="A68" s="3"/>
     </row>
     <row r="69" spans="1:1">
-      <c r="A69"/>
+      <c r="A69" s="3"/>
     </row>
     <row r="70" spans="1:1">
-      <c r="A70"/>
+      <c r="A70" s="3"/>
     </row>
     <row r="71" spans="1:1">
-      <c r="A71"/>
+      <c r="A71" s="3"/>
     </row>
     <row r="72" spans="1:1">
-      <c r="A72" s="1"/>
+      <c r="A72" s="3"/>
     </row>
     <row r="73" spans="1:1">
-      <c r="A73" s="1"/>
+      <c r="A73" s="3"/>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="1"/>
+      <c r="A74" s="3"/>
     </row>
     <row r="75" spans="1:1">
-      <c r="A75" s="1"/>
+      <c r="A75" s="3"/>
     </row>
     <row r="76" spans="1:1">
-      <c r="A76" s="1"/>
+      <c r="A76" s="3"/>
     </row>
     <row r="77" spans="1:1">
-      <c r="A77" s="1"/>
+      <c r="A77" s="3"/>
     </row>
     <row r="78" spans="1:1">
-      <c r="A78" s="1"/>
+      <c r="A78" s="3"/>
     </row>
     <row r="79" spans="1:1">
-      <c r="A79" s="1"/>
+      <c r="A79" s="3"/>
     </row>
     <row r="80" spans="1:1">
-      <c r="A80" s="1"/>
+      <c r="A80" s="3"/>
     </row>
     <row r="81" spans="1:1">
-      <c r="A81" s="1"/>
+      <c r="A81" s="3"/>
     </row>
     <row r="82" spans="1:1">
-      <c r="A82" s="1"/>
+      <c r="A82" s="3"/>
     </row>
     <row r="83" spans="1:1">
-      <c r="A83" s="1"/>
+      <c r="A83" s="3"/>
     </row>
     <row r="84" spans="1:1">
-      <c r="A84" s="1"/>
+      <c r="A84" s="3"/>
     </row>
     <row r="85" spans="1:1">
-      <c r="A85" s="1"/>
+      <c r="A85" s="3"/>
     </row>
     <row r="86" spans="1:1">
-      <c r="A86" s="1"/>
+      <c r="A86" s="3"/>
     </row>
     <row r="87" spans="1:1">
-      <c r="A87" s="1"/>
+      <c r="A87" s="3"/>
     </row>
     <row r="88" spans="1:1">
-      <c r="A88" s="1"/>
+      <c r="A88" s="3"/>
     </row>
     <row r="89" spans="1:1">
-      <c r="A89" s="1"/>
+      <c r="A89" s="3"/>
     </row>
     <row r="90" spans="1:1">
-      <c r="A90" s="1"/>
+      <c r="A90" s="3"/>
     </row>
     <row r="91" spans="1:1">
-      <c r="A91" s="1"/>
+      <c r="A91" s="3"/>
     </row>
     <row r="92" spans="1:1">
-      <c r="A92" s="1"/>
+      <c r="A92" s="3"/>
     </row>
     <row r="93" spans="1:1">
-      <c r="A93" s="1"/>
+      <c r="A93" s="3"/>
     </row>
     <row r="94" spans="1:1">
-      <c r="A94" s="1"/>
+      <c r="A94" s="3"/>
     </row>
     <row r="95" spans="1:1">
-      <c r="A95" s="1"/>
+      <c r="A95" s="3"/>
     </row>
     <row r="96" spans="1:1">
-      <c r="A96" s="1"/>
+      <c r="A96" s="3"/>
     </row>
     <row r="97" spans="1:1">
-      <c r="A97" s="1"/>
+      <c r="A97" s="3"/>
     </row>
     <row r="98" spans="1:1">
-      <c r="A98" s="1"/>
+      <c r="A98" s="3"/>
     </row>
     <row r="99" spans="1:1">
-      <c r="A99" s="1"/>
+      <c r="A99" s="3"/>
     </row>
     <row r="100" spans="1:1">
-      <c r="A100" s="1"/>
+      <c r="A100" s="3"/>
     </row>
     <row r="101" spans="1:1">
-      <c r="A101" s="1"/>
+      <c r="A101" s="3"/>
     </row>
     <row r="102" spans="1:1">
-      <c r="A102" s="1"/>
+      <c r="A102" s="3"/>
     </row>
     <row r="103" spans="1:1">
-      <c r="A103" s="1"/>
+      <c r="A103" s="3"/>
     </row>
     <row r="104" spans="1:1">
-      <c r="A104" s="1"/>
+      <c r="A104" s="3"/>
     </row>
     <row r="105" spans="1:1">
-      <c r="A105" s="1"/>
+      <c r="A105" s="3"/>
     </row>
     <row r="106" spans="1:1">
-      <c r="A106" s="1"/>
+      <c r="A106" s="3"/>
     </row>
     <row r="107" spans="1:1">
-      <c r="A107" s="1"/>
+      <c r="A107" s="3"/>
     </row>
     <row r="108" spans="1:1">
-      <c r="A108" s="1"/>
+      <c r="A108" s="3"/>
     </row>
     <row r="109" spans="1:1">
-      <c r="A109" s="1"/>
+      <c r="A109" s="3"/>
     </row>
     <row r="110" spans="1:1">
-      <c r="A110" s="1"/>
+      <c r="A110" s="3"/>
     </row>
     <row r="111" spans="1:1">
-      <c r="A111" s="1"/>
+      <c r="A111" s="3"/>
     </row>
     <row r="112" spans="1:1">
-      <c r="A112" s="1"/>
+      <c r="A112" s="3"/>
     </row>
     <row r="113" spans="1:1">
-      <c r="A113" s="1"/>
+      <c r="A113" s="3"/>
     </row>
     <row r="114" spans="1:1">
-      <c r="A114" s="1"/>
+      <c r="A114" s="3"/>
     </row>
     <row r="115" spans="1:1">
-      <c r="A115" s="1"/>
+      <c r="A115" s="3"/>
     </row>
     <row r="116" spans="1:1">
-      <c r="A116" s="1"/>
+      <c r="A116" s="3"/>
     </row>
     <row r="117" spans="1:1">
-      <c r="A117" s="1"/>
+      <c r="A117" s="3"/>
     </row>
     <row r="118" spans="1:1">
-      <c r="A118" s="1"/>
+      <c r="A118" s="3"/>
     </row>
     <row r="119" spans="1:1">
-      <c r="A119" s="1"/>
+      <c r="A119" s="3"/>
     </row>
     <row r="120" spans="1:1">
-      <c r="A120" s="1"/>
+      <c r="A120" s="3"/>
     </row>
     <row r="121" spans="1:1">
-      <c r="A121" s="1"/>
+      <c r="A121" s="3"/>
     </row>
     <row r="122" spans="1:1">
-      <c r="A122" s="1"/>
+      <c r="A122" s="3"/>
     </row>
     <row r="123" spans="1:1">
-      <c r="A123" s="1"/>
+      <c r="A123" s="3"/>
     </row>
     <row r="124" spans="1:1">
-      <c r="A124" s="1"/>
+      <c r="A124" s="3"/>
     </row>
     <row r="125" spans="1:1">
-      <c r="A125" s="1"/>
+      <c r="A125" s="3"/>
     </row>
     <row r="126" spans="1:1">
-      <c r="A126" s="1"/>
+      <c r="A126" s="3"/>
     </row>
     <row r="127" spans="1:1">
-      <c r="A127" s="1"/>
+      <c r="A127" s="3"/>
     </row>
     <row r="128" spans="1:1">
-      <c r="A128" s="1"/>
+      <c r="A128" s="3"/>
     </row>
     <row r="129" spans="1:1">
-      <c r="A129" s="1"/>
+      <c r="A129" s="3"/>
     </row>
     <row r="130" spans="1:1">
-      <c r="A130" s="1"/>
+      <c r="A130" s="3"/>
     </row>
     <row r="131" spans="1:1">
-      <c r="A131" s="1"/>
+      <c r="A131" s="3"/>
     </row>
     <row r="132" spans="1:1">
-      <c r="A132" s="1"/>
+      <c r="A132" s="3"/>
     </row>
     <row r="133" spans="1:1">
-      <c r="A133" s="1"/>
+      <c r="A133" s="3"/>
     </row>
     <row r="134" spans="1:1">
-      <c r="A134" s="1"/>
+      <c r="A134" s="3"/>
     </row>
     <row r="135" spans="1:1">
-      <c r="A135" s="1"/>
+      <c r="A135" s="3"/>
     </row>
     <row r="136" spans="1:1">
-      <c r="A136" s="1"/>
+      <c r="A136" s="3"/>
     </row>
     <row r="137" spans="1:1">
-      <c r="A137" s="1"/>
+      <c r="A137" s="3"/>
     </row>
     <row r="138" spans="1:1">
-      <c r="A138" s="1"/>
+      <c r="A138" s="3"/>
     </row>
     <row r="139" spans="1:1">
-      <c r="A139" s="1"/>
+      <c r="A139" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1975,7 +2345,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1776886078" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1777497327" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -1984,16 +2354,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1776886078" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1776886078" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1776886078" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1776886078" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1777497327" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1777497327" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1777497327" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1777497327" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1776886078" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777497327" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>

<commit_message>
Refatora testes utilizando Page Object Model
</commit_message>
<xml_diff>
--- a/docs/casos-de-teste-e2e.xlsx
+++ b/docs/casos-de-teste-e2e.xlsx
@@ -13,17 +13,17 @@
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1777497327" val="982" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1777497327" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1777497327" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1777497327"/>
+      <pm:revision xmlns:pm="smNativeData" day="1778179417" val="982" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1778179417" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1778179417" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1778179417"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="67">
   <si>
     <t>CASO DE TESTE</t>
   </si>
@@ -281,6 +281,18 @@
   </si>
   <si>
     <t>retorna à pagina inicial</t>
+  </si>
+  <si>
+    <t>acessa pagina inicial pelo menu superior</t>
+  </si>
+  <si>
+    <t>- acessar o site
+- logar conta
+- acessar lista de compras
+- clicar "home"</t>
+  </si>
+  <si>
+    <t>usuario é direcionado à pagina inicial</t>
   </si>
 </sst>
 </file>
@@ -307,7 +319,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777497327" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778179417" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -323,7 +335,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777497327" fgClr="FFFFFF" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778179417" fgClr="FFFFFF" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -338,7 +350,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1777497327" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1778179417" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -347,23 +359,12 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDEDEDE"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none"/>
@@ -374,7 +375,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -385,7 +386,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -396,7 +397,29 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="100" fgClr="00666666" bgLvl="0" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEDEDE"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEDEDE"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -407,7 +430,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -418,21 +452,29 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEDEDE"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
+          </ext>
+        </extLst>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -443,35 +485,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -482,7 +496,18 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+          </ext>
+        </extLst>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFFFFFFF"/>
+        <extLst>
+          <ext uri="smNativeData">
+            <pm:shade xmlns:pm="smNativeData" id="1778179417" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -490,41 +515,8 @@
     <fill>
       <patternFill patternType="none"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDEDEDE"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDEDEDE"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1777497327" type="1" fgLvl="13" fgClr="00000000" bgLvl="87" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="20">
+  <borders count="16">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -540,7 +532,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327"/>
+          <pm:border xmlns:pm="smNativeData" id="1778179417"/>
         </ext>
       </extLst>
     </border>
@@ -559,7 +551,100 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="double">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
+            <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="double">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
+            <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="double">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
+            <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -578,12 +663,35 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
+      <bottom style="none">
         <color rgb="FF000000"/>
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -593,206 +701,21 @@
       </extLst>
     </border>
     <border>
-      <left style="double">
+      <left style="none">
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="double">
+      <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="none">
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="double">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="double">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="double">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="2" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -810,36 +733,12 @@
       <top style="none">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
+      <bottom style="none">
         <color rgb="FF000000"/>
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -850,79 +749,18 @@
       <left style="none">
         <color rgb="FF000000"/>
       </left>
-      <right style="none">
+      <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="none">
+      <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="none">
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
-            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-          </pm:border>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -931,10 +769,10 @@
       </extLst>
     </border>
     <border>
-      <left style="thin">
+      <left style="none">
         <color rgb="FF000000"/>
       </left>
-      <right style="thin">
+      <right style="none">
         <color rgb="FF000000"/>
       </right>
       <top style="none">
@@ -945,7 +783,46 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
+          <pm:border xmlns:pm="smNativeData" id="1778179417"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="none">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="none">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417"/>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -962,14 +839,36 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
+      <bottom style="none">
         <color rgb="FF000000"/>
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1777497327">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
-            <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+          </pm:border>
+        </ext>
+      </extLst>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="none">
+        <color rgb="FF000000"/>
+      </bottom>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:border xmlns:pm="smNativeData" id="1778179417">
+            <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
+            <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -979,7 +878,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -991,16 +890,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1009,9 +911,6 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1027,61 +926,70 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="14" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="20" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1091,10 +999,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1777497327" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1778179417" count="1">
         <pm:charStyle name="Normal" fontId="0"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1777497327" count="3">
+      <pm:colors xmlns:pm="smNativeData" id="1778179417" count="3">
         <pm:color name="Cor 24" rgb="919191"/>
         <pm:color name="Cor 25" rgb="D9D9D9"/>
         <pm:color name="Cor 26" rgb="DEDEDE"/>
@@ -1360,7 +1268,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:XFD139"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="9" defaultColWidth="10.000000" defaultRowHeight="13.45"/>
   <cols>
     <col min="1" max="1" width="16.945946" customWidth="1" style="0"/>
@@ -1374,7 +1282,7 @@
     <col min="9" max="16384" width="10.000000" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16384" ht="29.25" customHeight="1">
+    <row r="1" spans="1:8" ht="29.25" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1401,10 +1309,10 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="67.85" customHeight="1">
-      <c r="A2" s="32" t="n">
+      <c r="A2" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="29" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -1427,10 +1335,10 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="63.70" customHeight="1">
-      <c r="A3" s="32" t="n">
+      <c r="A3" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="29" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="5" t="s">
@@ -1453,10 +1361,10 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="32" t="n">
+      <c r="A4" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="5" t="s">
@@ -1479,10 +1387,10 @@
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="32" t="n">
+      <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="29" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1505,10 +1413,10 @@
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="32" t="n">
+      <c r="A6" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="29" t="s">
         <v>24</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -1531,10 +1439,10 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="63.45" customHeight="1">
-      <c r="A7" s="32" t="n">
+      <c r="A7" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="29" t="s">
         <v>27</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -1557,20 +1465,20 @@
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="33"/>
-      <c r="B8" s="26"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="32" t="n">
+      <c r="A9" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="28" t="s">
         <v>30</v>
       </c>
       <c r="C9" s="5" t="s">
@@ -1593,10 +1501,10 @@
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="32" t="n">
+      <c r="A10" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="28" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -1619,10 +1527,10 @@
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="32" t="n">
+      <c r="A11" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="28" t="s">
         <v>37</v>
       </c>
       <c r="C11" s="5" t="s">
@@ -1645,10 +1553,10 @@
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="32" t="n">
+      <c r="A12" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="28" t="s">
         <v>24</v>
       </c>
       <c r="C12" s="5" t="s">
@@ -1671,10 +1579,10 @@
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="32" t="n">
+      <c r="A13" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="28" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="5" t="s">
@@ -1697,7 +1605,7 @@
       </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="33"/>
+      <c r="A14" s="27"/>
       <c r="B14" s="19"/>
       <c r="C14" s="20"/>
       <c r="D14" s="8"/>
@@ -1707,10 +1615,10 @@
       <c r="H14" s="8"/>
     </row>
     <row r="15" spans="1:8" ht="74.75" customHeight="1">
-      <c r="A15" s="29" t="n">
+      <c r="A15" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="25" t="s">
         <v>42</v>
       </c>
       <c r="C15" s="5" t="s">
@@ -1733,10 +1641,10 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="59.60" customHeight="1">
-      <c r="A16" s="30" t="n">
+      <c r="A16" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="25" t="s">
         <v>46</v>
       </c>
       <c r="C16" s="18" t="s">
@@ -1759,10 +1667,10 @@
       </c>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="30" t="n">
+      <c r="A17" s="24" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="25" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -1785,10 +1693,10 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="55.40" customHeight="1">
-      <c r="A18" s="30" t="n">
+      <c r="A18" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="25" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="5" t="s">
@@ -1811,10 +1719,10 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A19" s="30" t="n">
+      <c r="A19" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="25" t="s">
         <v>55</v>
       </c>
       <c r="C19" s="5" t="s">
@@ -1837,10 +1745,10 @@
       </c>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="30" t="n">
+      <c r="A20" s="24" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="25" t="s">
         <v>58</v>
       </c>
       <c r="C20" s="5" t="s">
@@ -1863,68 +1771,84 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A21" s="30" t="n">
+      <c r="A21" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="37" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A22" s="21"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
+    <row r="22" spans="1:8" ht="57.45" customHeight="1">
+      <c r="A22" s="30" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="G22" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="33" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A23" s="21"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-    </row>
-    <row r="24" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A24" s="25"/>
-    </row>
-    <row r="25" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A25" s="25"/>
-    </row>
-    <row r="26" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A26" s="25"/>
-    </row>
-    <row r="27" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A27" s="21"/>
-    </row>
-    <row r="28" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A28" s="21"/>
-    </row>
-    <row r="29" spans="1:8" ht="53.90" customHeight="1">
-      <c r="A29" s="21"/>
+      <c r="A23" s="14"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="1:1" ht="53.90" customHeight="1">
+      <c r="A24" s="1"/>
+    </row>
+    <row r="25" spans="1:1" ht="53.90" customHeight="1">
+      <c r="A25" s="1"/>
+    </row>
+    <row r="26" spans="1:1" ht="53.90" customHeight="1">
+      <c r="A26" s="1"/>
+    </row>
+    <row r="27" spans="1:1" ht="53.90" customHeight="1">
+      <c r="A27" s="14"/>
+    </row>
+    <row r="28" spans="1:1" ht="53.90" customHeight="1">
+      <c r="A28" s="14"/>
+    </row>
+    <row r="29" spans="1:1" ht="53.90" customHeight="1">
+      <c r="A29" s="14"/>
     </row>
     <row r="30" spans="1:8" ht="53.90" customHeight="1">
       <c r="A30" s="14"/>
@@ -2345,7 +2269,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1777497327" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1778179417" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2354,16 +2278,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1777497327" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1777497327" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1777497327" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1777497327" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1778179417" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1778179417" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1778179417" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1778179417" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1777497327" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1778179417" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>